<commit_message>
cambiando el presupuesto de computo/es raro este cambio ver primero
</commit_message>
<xml_diff>
--- a/Computo y Presupuesto -Segovia Joaquin.xlsx
+++ b/Computo y Presupuesto -Segovia Joaquin.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea Fernandez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea Fernandez\Documents\Pragma\presupuestador-obras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7D7FD5-9DEC-4DB5-9014-90FEE292D6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9110EE5-AC96-4F47-B543-B04BCE7E16ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3377,6 +3377,37 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="67" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="38" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3393,37 +3424,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="38" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1"/>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="Euro" xfId="7" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -3808,14 +3808,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="338" t="s">
+      <c r="A1" s="333" t="s">
         <v>345</v>
       </c>
-      <c r="B1" s="339"/>
-      <c r="C1" s="339"/>
-      <c r="D1" s="339"/>
-      <c r="E1" s="339"/>
-      <c r="F1" s="340"/>
+      <c r="B1" s="334"/>
+      <c r="C1" s="334"/>
+      <c r="D1" s="334"/>
+      <c r="E1" s="334"/>
+      <c r="F1" s="335"/>
     </row>
     <row r="2" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2"/>
@@ -3826,14 +3826,14 @@
       <c r="F2"/>
     </row>
     <row r="3" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A3" s="341" t="s">
+      <c r="A3" s="336" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="342"/>
-      <c r="C3" s="342"/>
-      <c r="D3" s="342"/>
-      <c r="E3" s="342"/>
-      <c r="F3" s="343"/>
+      <c r="B3" s="337"/>
+      <c r="C3" s="337"/>
+      <c r="D3" s="337"/>
+      <c r="E3" s="337"/>
+      <c r="F3" s="338"/>
     </row>
     <row r="4" spans="1:7" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B4" s="57"/>
@@ -3844,11 +3844,11 @@
         <v>21</v>
       </c>
       <c r="B5" s="59"/>
-      <c r="C5" s="344" t="s">
+      <c r="C5" s="342" t="s">
         <v>346</v>
       </c>
-      <c r="D5" s="345"/>
-      <c r="E5" s="346"/>
+      <c r="D5" s="343"/>
+      <c r="E5" s="344"/>
       <c r="F5" s="59"/>
     </row>
     <row r="6" spans="1:7" s="61" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5413,14 +5413,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="338" t="s">
+      <c r="A1" s="333" t="s">
         <v>345</v>
       </c>
-      <c r="B1" s="339"/>
-      <c r="C1" s="339"/>
-      <c r="D1" s="339"/>
-      <c r="E1" s="339"/>
-      <c r="F1" s="340"/>
+      <c r="B1" s="334"/>
+      <c r="C1" s="334"/>
+      <c r="D1" s="334"/>
+      <c r="E1" s="334"/>
+      <c r="F1" s="335"/>
     </row>
     <row r="2" spans="1:21" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2"/>
@@ -5431,26 +5431,26 @@
       <c r="F2"/>
     </row>
     <row r="3" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="341" t="s">
+      <c r="A3" s="336" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="342"/>
-      <c r="C3" s="342"/>
-      <c r="D3" s="342"/>
-      <c r="E3" s="342"/>
-      <c r="F3" s="343"/>
+      <c r="B3" s="337"/>
+      <c r="C3" s="337"/>
+      <c r="D3" s="337"/>
+      <c r="E3" s="337"/>
+      <c r="F3" s="338"/>
     </row>
     <row r="4" spans="1:21" ht="22.8" x14ac:dyDescent="0.4">
       <c r="A4" s="74"/>
     </row>
     <row r="5" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="347" t="s">
+      <c r="B5" s="339" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="348"/>
-      <c r="D5" s="348"/>
-      <c r="E5" s="348"/>
-      <c r="F5" s="349"/>
+      <c r="C5" s="340"/>
+      <c r="D5" s="340"/>
+      <c r="E5" s="340"/>
+      <c r="F5" s="341"/>
       <c r="G5" s="78"/>
       <c r="U5" s="79">
         <v>333</v>
@@ -13476,7 +13476,7 @@
         <v>28</v>
       </c>
       <c r="G452" s="89"/>
-      <c r="H452" s="350" t="s">
+      <c r="H452" s="332" t="s">
         <v>564</v>
       </c>
     </row>
@@ -41293,7 +41293,7 @@
         <v>359</v>
       </c>
       <c r="K9">
-        <f t="shared" ref="K7:K20" si="0">G9*H9*I9</f>
+        <f t="shared" ref="K9:K20" si="0">G9*H9*I9</f>
         <v>0.16000000000000003</v>
       </c>
       <c r="L9" s="328"/>
@@ -44406,14 +44406,14 @@
       <c r="D3" s="269"/>
     </row>
     <row r="4" spans="2:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="C4" s="332" t="s">
+      <c r="C4" s="345" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="332"/>
-      <c r="E4" s="332"/>
-      <c r="F4" s="332"/>
-      <c r="G4" s="332"/>
-      <c r="H4" s="332"/>
+      <c r="D4" s="345"/>
+      <c r="E4" s="345"/>
+      <c r="F4" s="345"/>
+      <c r="G4" s="345"/>
+      <c r="H4" s="345"/>
       <c r="I4" s="268"/>
       <c r="J4" s="1"/>
     </row>
@@ -44429,13 +44429,13 @@
     </row>
     <row r="6" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C6" s="280"/>
-      <c r="D6" s="335" t="s">
+      <c r="D6" s="348" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="336"/>
-      <c r="F6" s="336"/>
-      <c r="G6" s="336"/>
-      <c r="H6" s="337"/>
+      <c r="E6" s="349"/>
+      <c r="F6" s="349"/>
+      <c r="G6" s="349"/>
+      <c r="H6" s="350"/>
       <c r="I6" s="268"/>
       <c r="J6" s="1"/>
     </row>
@@ -44458,8 +44458,8 @@
       <c r="H8" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="I8" s="333"/>
-      <c r="J8" s="334"/>
+      <c r="I8" s="346"/>
+      <c r="J8" s="347"/>
     </row>
     <row r="9" spans="2:11" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C9" s="282"/>

</xml_diff>